<commit_message>
Jornada 8: análisis visual del resumen oficial
</commit_message>
<xml_diff>
--- a/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
+++ b/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
@@ -43,7 +43,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'partidos_rivales'!$A$1:$H$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'goles_video'!$A$1:$Z$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'resumenes_youtube'!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'resumenes_youtube'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'jugadores'!$A$1:$I$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'minutos_partido'!$A$1:$F$129</definedName>
   </definedNames>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21">
@@ -30481,12 +30481,12 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>No se ha podido acceder a un vídeo reproducible ni verificar sus fotogramas</t>
+          <t>El acceso directo de YouTube fallaba; el usuario ha facilitado el archivo del resumen oficial (154,6 s)</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Análisis visual pendiente; no se modifica goles_video.csv (partido 0-0)</t>
+          <t>Análisis visual completado el 19-10-2026; no contiene el córner final al larguero; no se modifica goles_video.csv</t>
         </is>
       </c>
     </row>
@@ -33513,7 +33513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33826,8 +33826,41 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Real Murcia</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Real Federación Española Fútbol</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Resumen #PrimeraFederación | Real Murcia CF 0-0 Real Zaragoza | Jornada 8 | Temporada 2026/2027</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>2:35</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Eq-htl0RmVs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G9"/>
+  <autoFilter ref="A1:G10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -33837,6 +33870,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Incorporar 41 estadísticas de Murcia-Zaragoza contrastadas con capturas de Sofascore
</commit_message>
<xml_diff>
--- a/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
+++ b/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
@@ -36,7 +36,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'tarjetas'!$A$1:$E$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'tiros'!$A$1:$J$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'estadisticas'!$A$1:$G$159</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'sofascore'!$A$1:$F$263</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'sofascore'!$A$1:$F$304</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'grupo2_partidos'!$A$1:$AO$141</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'clasificacion'!$A$1:$K$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'proximos'!$A$1:$F$4</definedName>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>262</v>
+        <v>303</v>
       </c>
     </row>
     <row r="14">
@@ -812,12 +812,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F263"/>
+  <dimension ref="A1:F304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
@@ -7143,8 +7143,992 @@
         </is>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B264" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C264" s="4" t="inlineStr">
+        <is>
+          <t>posesion_pct</t>
+        </is>
+      </c>
+      <c r="D264" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="E264" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="F264" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B265" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C265" s="5" t="inlineStr">
+        <is>
+          <t>xg</t>
+        </is>
+      </c>
+      <c r="D265" s="5" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="E265" s="5" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="F265" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B266" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C266" s="4" t="inlineStr">
+        <is>
+          <t>tiros</t>
+        </is>
+      </c>
+      <c r="D266" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E266" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F266" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B267" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C267" s="5" t="inlineStr">
+        <is>
+          <t>tiros_a_puerta</t>
+        </is>
+      </c>
+      <c r="D267" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E267" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F267" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B268" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C268" s="4" t="inlineStr">
+        <is>
+          <t>xgot</t>
+        </is>
+      </c>
+      <c r="D268" s="4" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E268" s="4" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F268" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B269" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C269" s="5" t="inlineStr">
+        <is>
+          <t>tiros_al_palo</t>
+        </is>
+      </c>
+      <c r="D269" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E269" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F269" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B270" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C270" s="4" t="inlineStr">
+        <is>
+          <t>tiros_fuera</t>
+        </is>
+      </c>
+      <c r="D270" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E270" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F270" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B271" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C271" s="5" t="inlineStr">
+        <is>
+          <t>tiros_bloqueados</t>
+        </is>
+      </c>
+      <c r="D271" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E271" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F271" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B272" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C272" s="4" t="inlineStr">
+        <is>
+          <t>tiros_dentro_area</t>
+        </is>
+      </c>
+      <c r="D272" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E272" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F272" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B273" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C273" s="5" t="inlineStr">
+        <is>
+          <t>tiros_fuera_area</t>
+        </is>
+      </c>
+      <c r="D273" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E273" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F273" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B274" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C274" s="4" t="inlineStr">
+        <is>
+          <t>corners</t>
+        </is>
+      </c>
+      <c r="D274" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E274" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F274" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B275" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C275" s="5" t="inlineStr">
+        <is>
+          <t>pases</t>
+        </is>
+      </c>
+      <c r="D275" s="5" t="n">
+        <v>379</v>
+      </c>
+      <c r="E275" s="5" t="n">
+        <v>394</v>
+      </c>
+      <c r="F275" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B276" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C276" s="4" t="inlineStr">
+        <is>
+          <t>pases_buenos</t>
+        </is>
+      </c>
+      <c r="D276" s="4" t="n">
+        <v>302</v>
+      </c>
+      <c r="E276" s="4" t="n">
+        <v>306</v>
+      </c>
+      <c r="F276" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B277" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C277" s="5" t="inlineStr">
+        <is>
+          <t>faltas</t>
+        </is>
+      </c>
+      <c r="D277" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E277" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="F277" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B278" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C278" s="4" t="inlineStr">
+        <is>
+          <t>amarillas</t>
+        </is>
+      </c>
+      <c r="D278" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E278" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F278" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B279" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C279" s="5" t="inlineStr">
+        <is>
+          <t>rojas</t>
+        </is>
+      </c>
+      <c r="D279" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E279" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F279" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B280" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C280" s="4" t="inlineStr">
+        <is>
+          <t>entradas</t>
+        </is>
+      </c>
+      <c r="D280" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E280" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="F280" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B281" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C281" s="5" t="inlineStr">
+        <is>
+          <t>tiros_libres</t>
+        </is>
+      </c>
+      <c r="D281" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="E281" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="F281" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B282" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C282" s="4" t="inlineStr">
+        <is>
+          <t>faltas_recibidas_ultimo_tercio</t>
+        </is>
+      </c>
+      <c r="D282" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E282" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F282" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B283" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C283" s="5" t="inlineStr">
+        <is>
+          <t>fueras_juego</t>
+        </is>
+      </c>
+      <c r="D283" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E283" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F283" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B284" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C284" s="4" t="inlineStr">
+        <is>
+          <t>saques_banda</t>
+        </is>
+      </c>
+      <c r="D284" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E284" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="F284" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B285" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C285" s="5" t="inlineStr">
+        <is>
+          <t>pases_ultimo_tercio</t>
+        </is>
+      </c>
+      <c r="D285" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="E285" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F285" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B286" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C286" s="4" t="inlineStr">
+        <is>
+          <t>balones_largos_ok</t>
+        </is>
+      </c>
+      <c r="D286" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E286" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="F286" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B287" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C287" s="5" t="inlineStr">
+        <is>
+          <t>balones_largos_total</t>
+        </is>
+      </c>
+      <c r="D287" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="E287" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="F287" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B288" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C288" s="4" t="inlineStr">
+        <is>
+          <t>centros_ok</t>
+        </is>
+      </c>
+      <c r="D288" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E288" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F288" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B289" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C289" s="5" t="inlineStr">
+        <is>
+          <t>centros_total</t>
+        </is>
+      </c>
+      <c r="D289" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="E289" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="F289" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B290" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C290" s="4" t="inlineStr">
+        <is>
+          <t>duelos_ganados_pct</t>
+        </is>
+      </c>
+      <c r="D290" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="E290" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="F290" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B291" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C291" s="5" t="inlineStr">
+        <is>
+          <t>desposeido</t>
+        </is>
+      </c>
+      <c r="D291" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="E291" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="F291" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B292" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C292" s="4" t="inlineStr">
+        <is>
+          <t>duelos_suelo_ok</t>
+        </is>
+      </c>
+      <c r="D292" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="E292" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="F292" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B293" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C293" s="5" t="inlineStr">
+        <is>
+          <t>duelos_suelo_total</t>
+        </is>
+      </c>
+      <c r="D293" s="5" t="n">
+        <v>81</v>
+      </c>
+      <c r="E293" s="5" t="n">
+        <v>81</v>
+      </c>
+      <c r="F293" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B294" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C294" s="4" t="inlineStr">
+        <is>
+          <t>duelos_aereos_ok</t>
+        </is>
+      </c>
+      <c r="D294" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E294" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F294" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B295" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C295" s="5" t="inlineStr">
+        <is>
+          <t>duelos_aereos_total</t>
+        </is>
+      </c>
+      <c r="D295" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="E295" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F295" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B296" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C296" s="4" t="inlineStr">
+        <is>
+          <t>regates_ok</t>
+        </is>
+      </c>
+      <c r="D296" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E296" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F296" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B297" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C297" s="5" t="inlineStr">
+        <is>
+          <t>regates_total</t>
+        </is>
+      </c>
+      <c r="D297" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E297" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F297" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B298" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C298" s="4" t="inlineStr">
+        <is>
+          <t>entradas_ganadas_pct</t>
+        </is>
+      </c>
+      <c r="D298" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="E298" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="F298" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B299" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C299" s="5" t="inlineStr">
+        <is>
+          <t>intercepciones</t>
+        </is>
+      </c>
+      <c r="D299" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E299" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F299" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B300" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C300" s="4" t="inlineStr">
+        <is>
+          <t>recuperaciones</t>
+        </is>
+      </c>
+      <c r="D300" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="E300" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="F300" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B301" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C301" s="5" t="inlineStr">
+        <is>
+          <t>despejes</t>
+        </is>
+      </c>
+      <c r="D301" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E301" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="F301" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B302" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C302" s="4" t="inlineStr">
+        <is>
+          <t>paradas</t>
+        </is>
+      </c>
+      <c r="D302" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E302" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F302" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B303" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C303" s="5" t="inlineStr">
+        <is>
+          <t>goles_evitados</t>
+        </is>
+      </c>
+      <c r="D303" s="5" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E303" s="5" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F303" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B304" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C304" s="4" t="inlineStr">
+        <is>
+          <t>saques_meta</t>
+        </is>
+      </c>
+      <c r="D304" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E304" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F304" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F263"/>
+  <autoFilter ref="A1:F304"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
@@ -7408,6 +8392,47 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F261" r:id="rId260"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F262" r:id="rId261"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F267" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F268" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F269" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F270" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F271" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F272" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F273" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F274" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F275" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F276" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F277" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F278" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F279" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F291" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F292" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F293" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F294" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F295" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F296" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F297" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F298" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F299" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F300" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F301" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F302" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F303" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F304" r:id="rId303"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -30366,7 +31391,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>No añado métricas ni filas del grupo sin respuesta de la fuente; cobertura de grupo 2 permanece hasta J7</t>
+          <t>Métricas de Murcia-Zaragoza incorporadas el 20-10-2026 mediante capturas de Sofascore facilitadas por el usuario; comparación del grupo con corte común J7 mientras faltan los otros nueve partidos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Completar jornada 8 del grupo 2 y recalcular estadísticas y gráficos
</commit_message>
<xml_diff>
--- a/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
+++ b/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
@@ -37,7 +37,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'tiros'!$A$1:$J$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'estadisticas'!$A$1:$G$159</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'sofascore'!$A$1:$F$304</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'grupo2_partidos'!$A$1:$AO$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'grupo2_partidos'!$A$1:$AO$161</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'clasificacion'!$A$1:$K$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'proximos'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'partidos_rivales'!$A$1:$H$16</definedName>
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>140</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15">
@@ -8444,7 +8444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO141"/>
+  <dimension ref="A1:AO161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -27149,8 +27149,2556 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B142" s="4" t="n"/>
+      <c r="C142" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>Cartagena</t>
+        </is>
+      </c>
+      <c r="E142" s="4" t="inlineStr">
+        <is>
+          <t>CE Europa</t>
+        </is>
+      </c>
+      <c r="F142" s="4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G142" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H142" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I142" s="4" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="J142" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K142" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L142" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M142" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="N142" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="O142" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P142" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q142" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="R142" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S142" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="T142" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="U142" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="V142" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="W142" s="4" t="n">
+        <v>280</v>
+      </c>
+      <c r="X142" s="4" t="n">
+        <v>381</v>
+      </c>
+      <c r="Y142" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z142" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA142" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="AB142" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC142" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD142" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE142" s="4" t="n"/>
+      <c r="AF142" s="4" t="n"/>
+      <c r="AG142" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="AH142" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="AI142" s="4" t="n"/>
+      <c r="AJ142" s="4" t="n"/>
+      <c r="AK142" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="AL142" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="AM142" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN142" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO142" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B143" s="5" t="n"/>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>CE Europa</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>Cartagena</t>
+        </is>
+      </c>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="G143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I143" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J143" s="5" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="K143" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L143" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M143" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="N143" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="O143" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P143" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q143" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="R143" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="S143" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="T143" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="U143" s="5" t="n">
+        <v>448</v>
+      </c>
+      <c r="V143" s="5" t="n">
+        <v>355</v>
+      </c>
+      <c r="W143" s="5" t="n">
+        <v>381</v>
+      </c>
+      <c r="X143" s="5" t="n">
+        <v>280</v>
+      </c>
+      <c r="Y143" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z143" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA143" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB143" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="AC143" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE143" s="5" t="n"/>
+      <c r="AF143" s="5" t="n"/>
+      <c r="AG143" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="AH143" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="AI143" s="5" t="n"/>
+      <c r="AJ143" s="5" t="n"/>
+      <c r="AK143" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="AL143" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="AM143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN143" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO143" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B144" s="4" t="n"/>
+      <c r="C144" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="inlineStr">
+        <is>
+          <t>Alcorcón</t>
+        </is>
+      </c>
+      <c r="E144" s="4" t="inlineStr">
+        <is>
+          <t>SD Huesca</t>
+        </is>
+      </c>
+      <c r="F144" s="4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G144" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H144" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I144" s="4" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="J144" s="4" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="K144" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L144" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M144" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="N144" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="O144" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P144" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q144" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="R144" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S144" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="T144" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="U144" s="4" t="n">
+        <v>432</v>
+      </c>
+      <c r="V144" s="4" t="n">
+        <v>356</v>
+      </c>
+      <c r="W144" s="4" t="n">
+        <v>374</v>
+      </c>
+      <c r="X144" s="4" t="n">
+        <v>281</v>
+      </c>
+      <c r="Y144" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z144" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA144" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB144" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="AC144" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD144" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE144" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF144" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG144" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="AH144" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="AI144" s="4" t="n"/>
+      <c r="AJ144" s="4" t="n"/>
+      <c r="AK144" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="AL144" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="AM144" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN144" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO144" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B145" s="5" t="n"/>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>SD Huesca</t>
+        </is>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>Alcorcón</t>
+        </is>
+      </c>
+      <c r="F145" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="G145" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H145" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I145" s="5" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="J145" s="5" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="K145" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L145" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M145" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N145" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="O145" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="P145" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q145" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="R145" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="S145" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="T145" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="U145" s="5" t="n">
+        <v>356</v>
+      </c>
+      <c r="V145" s="5" t="n">
+        <v>432</v>
+      </c>
+      <c r="W145" s="5" t="n">
+        <v>281</v>
+      </c>
+      <c r="X145" s="5" t="n">
+        <v>374</v>
+      </c>
+      <c r="Y145" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z145" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA145" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="AB145" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC145" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD145" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE145" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF145" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG145" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="AH145" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="AI145" s="5" t="n"/>
+      <c r="AJ145" s="5" t="n"/>
+      <c r="AK145" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="AL145" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="AM145" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN145" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO145" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B146" s="4" t="n"/>
+      <c r="C146" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D146" s="4" t="inlineStr">
+        <is>
+          <t>CDA Águilas FC</t>
+        </is>
+      </c>
+      <c r="E146" s="4" t="inlineStr">
+        <is>
+          <t>UD Ibiza</t>
+        </is>
+      </c>
+      <c r="F146" s="4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G146" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H146" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I146" s="4" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J146" s="4" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="K146" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L146" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M146" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="N146" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O146" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P146" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q146" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="R146" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="S146" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="T146" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="U146" s="4" t="n">
+        <v>269</v>
+      </c>
+      <c r="V146" s="4" t="n">
+        <v>465</v>
+      </c>
+      <c r="W146" s="4" t="n">
+        <v>173</v>
+      </c>
+      <c r="X146" s="4" t="n">
+        <v>351</v>
+      </c>
+      <c r="Y146" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="Z146" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA146" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="AB146" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="AC146" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD146" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE146" s="4" t="n"/>
+      <c r="AF146" s="4" t="n"/>
+      <c r="AG146" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="AH146" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="AI146" s="4" t="n"/>
+      <c r="AJ146" s="4" t="n"/>
+      <c r="AK146" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="AL146" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="AM146" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN146" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO146" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B147" s="5" t="n"/>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>UD Ibiza</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>CDA Águilas FC</t>
+        </is>
+      </c>
+      <c r="F147" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="G147" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H147" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I147" s="5" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J147" s="5" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="K147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L147" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M147" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="N147" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="O147" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="P147" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q147" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="R147" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="S147" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="T147" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="U147" s="5" t="n">
+        <v>465</v>
+      </c>
+      <c r="V147" s="5" t="n">
+        <v>269</v>
+      </c>
+      <c r="W147" s="5" t="n">
+        <v>351</v>
+      </c>
+      <c r="X147" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="Y147" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z147" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="AA147" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="AB147" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="AC147" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD147" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE147" s="5" t="n"/>
+      <c r="AF147" s="5" t="n"/>
+      <c r="AG147" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="AH147" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="AI147" s="5" t="n"/>
+      <c r="AJ147" s="5" t="n"/>
+      <c r="AK147" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="AL147" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="AM147" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN147" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO147" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B148" s="4" t="n"/>
+      <c r="C148" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D148" s="4" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="E148" s="4" t="inlineStr">
+        <is>
+          <t>CD Teruel</t>
+        </is>
+      </c>
+      <c r="F148" s="4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G148" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H148" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I148" s="4" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="J148" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K148" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L148" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M148" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="N148" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O148" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P148" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q148" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="R148" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S148" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="T148" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="U148" s="4" t="n">
+        <v>563</v>
+      </c>
+      <c r="V148" s="4" t="n">
+        <v>358</v>
+      </c>
+      <c r="W148" s="4" t="n">
+        <v>484</v>
+      </c>
+      <c r="X148" s="4" t="n">
+        <v>263</v>
+      </c>
+      <c r="Y148" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z148" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA148" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="AB148" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC148" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD148" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE148" s="4" t="n"/>
+      <c r="AF148" s="4" t="n"/>
+      <c r="AG148" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="AH148" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="AI148" s="4" t="n"/>
+      <c r="AJ148" s="4" t="n"/>
+      <c r="AK148" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="AL148" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="AM148" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN148" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO148" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B149" s="5" t="n"/>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>CD Teruel</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="F149" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="G149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I149" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J149" s="5" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="K149" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L149" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M149" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="N149" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="O149" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="P149" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q149" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="R149" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="S149" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="T149" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="U149" s="5" t="n">
+        <v>358</v>
+      </c>
+      <c r="V149" s="5" t="n">
+        <v>563</v>
+      </c>
+      <c r="W149" s="5" t="n">
+        <v>263</v>
+      </c>
+      <c r="X149" s="5" t="n">
+        <v>484</v>
+      </c>
+      <c r="Y149" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z149" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA149" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB149" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="AC149" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD149" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE149" s="5" t="n"/>
+      <c r="AF149" s="5" t="n"/>
+      <c r="AG149" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="AH149" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="AI149" s="5" t="n"/>
+      <c r="AJ149" s="5" t="n"/>
+      <c r="AK149" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="AL149" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="AM149" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN149" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO149" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B150" s="4" t="n">
+        <v>16599924</v>
+      </c>
+      <c r="C150" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D150" s="4" t="inlineStr">
+        <is>
+          <t>Algeciras</t>
+        </is>
+      </c>
+      <c r="E150" s="4" t="inlineStr">
+        <is>
+          <t>Hércules</t>
+        </is>
+      </c>
+      <c r="F150" s="4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G150" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H150" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I150" s="4" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J150" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K150" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L150" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M150" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="N150" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O150" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P150" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q150" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R150" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S150" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="T150" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="U150" s="4" t="n">
+        <v>440</v>
+      </c>
+      <c r="V150" s="4" t="n">
+        <v>413</v>
+      </c>
+      <c r="W150" s="4" t="n">
+        <v>368</v>
+      </c>
+      <c r="X150" s="4" t="n">
+        <v>329</v>
+      </c>
+      <c r="Y150" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z150" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA150" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="AB150" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="AC150" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD150" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE150" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF150" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG150" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="AH150" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="AI150" s="4" t="n"/>
+      <c r="AJ150" s="4" t="n"/>
+      <c r="AK150" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="AL150" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="AM150" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN150" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO150" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es-la/football/match/algeciras-cf-hercules-cf/ChbsOOb#id:16599924,tab:statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B151" s="5" t="n">
+        <v>16599924</v>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>Hércules</t>
+        </is>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>Algeciras</t>
+        </is>
+      </c>
+      <c r="F151" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="G151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I151" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J151" s="5" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="K151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L151" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M151" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N151" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="O151" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P151" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q151" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="R151" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="S151" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="T151" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="U151" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="V151" s="5" t="n">
+        <v>440</v>
+      </c>
+      <c r="W151" s="5" t="n">
+        <v>329</v>
+      </c>
+      <c r="X151" s="5" t="n">
+        <v>368</v>
+      </c>
+      <c r="Y151" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z151" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA151" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="AB151" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="AC151" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD151" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE151" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG151" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="AH151" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="AI151" s="5" t="n"/>
+      <c r="AJ151" s="5" t="n"/>
+      <c r="AK151" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="AL151" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="AM151" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN151" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO151" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es-la/football/match/algeciras-cf-hercules-cf/ChbsOOb#id:16599924,tab:statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B152" s="4" t="n">
+        <v>16599937</v>
+      </c>
+      <c r="C152" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D152" s="4" t="inlineStr">
+        <is>
+          <t>Real Madrid Castilla</t>
+        </is>
+      </c>
+      <c r="E152" s="4" t="inlineStr">
+        <is>
+          <t>Antequera</t>
+        </is>
+      </c>
+      <c r="F152" s="4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G152" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H152" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I152" s="4" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="J152" s="4" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="K152" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L152" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M152" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N152" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="O152" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P152" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q152" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="R152" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S152" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="T152" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="U152" s="4" t="n">
+        <v>555</v>
+      </c>
+      <c r="V152" s="4" t="n">
+        <v>358</v>
+      </c>
+      <c r="W152" s="4" t="n">
+        <v>496</v>
+      </c>
+      <c r="X152" s="4" t="n">
+        <v>301</v>
+      </c>
+      <c r="Y152" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z152" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA152" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="AB152" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="AC152" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD152" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE152" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF152" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG152" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="AH152" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="AI152" s="4" t="n"/>
+      <c r="AJ152" s="4" t="n"/>
+      <c r="AK152" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="AL152" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="AM152" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN152" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO152" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es-la/football/match/antequera-real-madrid-castilla-u21/ubcsyLj#id:16599937,tab:statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B153" s="5" t="n">
+        <v>16599937</v>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>Antequera</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>Real Madrid Castilla</t>
+        </is>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="G153" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H153" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I153" s="5" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J153" s="5" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="K153" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L153" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M153" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="N153" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="O153" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P153" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q153" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="R153" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="S153" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="T153" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="U153" s="5" t="n">
+        <v>358</v>
+      </c>
+      <c r="V153" s="5" t="n">
+        <v>555</v>
+      </c>
+      <c r="W153" s="5" t="n">
+        <v>301</v>
+      </c>
+      <c r="X153" s="5" t="n">
+        <v>496</v>
+      </c>
+      <c r="Y153" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z153" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA153" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="AB153" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="AC153" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD153" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE153" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG153" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="AH153" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="AI153" s="5" t="n"/>
+      <c r="AJ153" s="5" t="n"/>
+      <c r="AK153" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="AL153" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="AM153" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN153" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO153" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es-la/football/match/antequera-real-madrid-castilla-u21/ubcsyLj#id:16599937,tab:statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B154" s="4" t="n">
+        <v>16599934</v>
+      </c>
+      <c r="C154" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>Gimnàstic</t>
+        </is>
+      </c>
+      <c r="E154" s="4" t="inlineStr">
+        <is>
+          <t>Atlético Madrileño</t>
+        </is>
+      </c>
+      <c r="F154" s="4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G154" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H154" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I154" s="4" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="J154" s="4" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="K154" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L154" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M154" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N154" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="O154" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P154" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q154" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R154" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S154" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="T154" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="U154" s="4" t="n">
+        <v>221</v>
+      </c>
+      <c r="V154" s="4" t="n">
+        <v>585</v>
+      </c>
+      <c r="W154" s="4" t="n">
+        <v>138</v>
+      </c>
+      <c r="X154" s="4" t="n">
+        <v>501</v>
+      </c>
+      <c r="Y154" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z154" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA154" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="AB154" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="AC154" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD154" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE154" s="4" t="n"/>
+      <c r="AF154" s="4" t="n"/>
+      <c r="AG154" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="AH154" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="AI154" s="4" t="n"/>
+      <c r="AJ154" s="4" t="n"/>
+      <c r="AK154" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="AL154" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="AM154" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN154" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO154" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es-la/football/match/atletico-madrileno-gimnastic-de-tarragona/PgbsBLj#id:16599934,tab:statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B155" s="5" t="n">
+        <v>16599934</v>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>Atlético Madrileño</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>Gimnàstic</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="G155" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H155" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I155" s="5" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="J155" s="5" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="K155" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L155" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M155" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="N155" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="O155" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="P155" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q155" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="R155" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="S155" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="T155" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="U155" s="5" t="n">
+        <v>585</v>
+      </c>
+      <c r="V155" s="5" t="n">
+        <v>221</v>
+      </c>
+      <c r="W155" s="5" t="n">
+        <v>501</v>
+      </c>
+      <c r="X155" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="Y155" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z155" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA155" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="AB155" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="AC155" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD155" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE155" s="5" t="n"/>
+      <c r="AF155" s="5" t="n"/>
+      <c r="AG155" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="AH155" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="AI155" s="5" t="n"/>
+      <c r="AJ155" s="5" t="n"/>
+      <c r="AK155" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="AL155" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="AM155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN155" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO155" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es-la/football/match/atletico-madrileno-gimnastic-de-tarragona/PgbsBLj#id:16599934,tab:statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B156" s="4" t="n">
+        <v>16599940</v>
+      </c>
+      <c r="C156" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>Sant Andreu</t>
+        </is>
+      </c>
+      <c r="E156" s="4" t="inlineStr">
+        <is>
+          <t>Juventud Torremolinos CF</t>
+        </is>
+      </c>
+      <c r="F156" s="4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G156" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H156" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I156" s="4" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="J156" s="4" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="K156" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L156" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M156" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="N156" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="O156" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="P156" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q156" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="R156" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S156" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="T156" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="U156" s="4" t="n">
+        <v>444</v>
+      </c>
+      <c r="V156" s="4" t="n">
+        <v>424</v>
+      </c>
+      <c r="W156" s="4" t="n">
+        <v>351</v>
+      </c>
+      <c r="X156" s="4" t="n">
+        <v>304</v>
+      </c>
+      <c r="Y156" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z156" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA156" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="AB156" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="AC156" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD156" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE156" s="4" t="n"/>
+      <c r="AF156" s="4" t="n"/>
+      <c r="AG156" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AH156" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AI156" s="4" t="n"/>
+      <c r="AJ156" s="4" t="n"/>
+      <c r="AK156" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="AL156" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="AM156" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AN156" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="AO156" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es-la/football/match/juventud-torremolinos-cf-ue-sant-andreu-u19/nMjshtfc#id:16599940,tab:statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B157" s="5" t="n">
+        <v>16599940</v>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>Juventud Torremolinos CF</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>Sant Andreu</t>
+        </is>
+      </c>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="G157" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H157" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I157" s="5" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="J157" s="5" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="K157" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L157" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M157" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="N157" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="O157" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="P157" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q157" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="R157" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="S157" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="T157" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="U157" s="5" t="n">
+        <v>424</v>
+      </c>
+      <c r="V157" s="5" t="n">
+        <v>444</v>
+      </c>
+      <c r="W157" s="5" t="n">
+        <v>304</v>
+      </c>
+      <c r="X157" s="5" t="n">
+        <v>351</v>
+      </c>
+      <c r="Y157" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z157" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA157" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="AB157" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="AC157" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD157" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE157" s="5" t="n"/>
+      <c r="AF157" s="5" t="n"/>
+      <c r="AG157" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="AH157" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="AI157" s="5" t="n"/>
+      <c r="AJ157" s="5" t="n"/>
+      <c r="AK157" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="AL157" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="AM157" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="AN157" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO157" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es-la/football/match/juventud-torremolinos-cf-ue-sant-andreu-u19/nMjshtfc#id:16599940,tab:statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B158" s="4" t="n">
+        <v>16599928</v>
+      </c>
+      <c r="C158" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>Real Jaén</t>
+        </is>
+      </c>
+      <c r="E158" s="4" t="inlineStr">
+        <is>
+          <t>Rayo Majadahonda</t>
+        </is>
+      </c>
+      <c r="F158" s="4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G158" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H158" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I158" s="4" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="J158" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K158" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L158" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M158" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N158" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="O158" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P158" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q158" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R158" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="S158" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="T158" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="U158" s="4" t="n">
+        <v>354</v>
+      </c>
+      <c r="V158" s="4" t="n">
+        <v>421</v>
+      </c>
+      <c r="W158" s="4" t="n">
+        <v>271</v>
+      </c>
+      <c r="X158" s="4" t="n">
+        <v>340</v>
+      </c>
+      <c r="Y158" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z158" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA158" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB158" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC158" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD158" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE158" s="4" t="n"/>
+      <c r="AF158" s="4" t="n"/>
+      <c r="AG158" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="AH158" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="AI158" s="4" t="n"/>
+      <c r="AJ158" s="4" t="n"/>
+      <c r="AK158" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="AL158" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="AM158" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="AN158" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO158" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es-la/football/match/rayo-majadahonda-real-jaen/QgbszQFb#id:16599928,tab:statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B159" s="5" t="n">
+        <v>16599928</v>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>Rayo Majadahonda</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>Real Jaén</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="G159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I159" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J159" s="5" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="K159" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="L159" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M159" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="N159" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="O159" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="P159" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q159" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="R159" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="S159" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="T159" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="U159" s="5" t="n">
+        <v>421</v>
+      </c>
+      <c r="V159" s="5" t="n">
+        <v>354</v>
+      </c>
+      <c r="W159" s="5" t="n">
+        <v>340</v>
+      </c>
+      <c r="X159" s="5" t="n">
+        <v>271</v>
+      </c>
+      <c r="Y159" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z159" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA159" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB159" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC159" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD159" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE159" s="5" t="n"/>
+      <c r="AF159" s="5" t="n"/>
+      <c r="AG159" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="AH159" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="AI159" s="5" t="n"/>
+      <c r="AJ159" s="5" t="n"/>
+      <c r="AK159" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="AL159" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="AM159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN159" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="AO159" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es-la/football/match/rayo-majadahonda-real-jaen/QgbszQFb#id:16599928,tab:statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B160" s="4" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C160" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>Real Murcia</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="inlineStr">
+        <is>
+          <t>Real Zaragoza</t>
+        </is>
+      </c>
+      <c r="F160" s="4" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G160" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I160" s="4" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J160" s="4" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="K160" s="4" t="n"/>
+      <c r="L160" s="4" t="n"/>
+      <c r="M160" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="N160" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="O160" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P160" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q160" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R160" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S160" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="T160" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="U160" s="4" t="n">
+        <v>394</v>
+      </c>
+      <c r="V160" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="W160" s="4" t="n">
+        <v>306</v>
+      </c>
+      <c r="X160" s="4" t="n">
+        <v>302</v>
+      </c>
+      <c r="Y160" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z160" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA160" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB160" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="AC160" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD160" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE160" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF160" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG160" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="AH160" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="AI160" s="4" t="n"/>
+      <c r="AJ160" s="4" t="n"/>
+      <c r="AK160" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="AL160" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="AM160" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN160" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO160" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B161" s="5" t="n">
+        <v>16599931</v>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>Real Zaragoza</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>Real Murcia</t>
+        </is>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="G161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I161" s="5" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="J161" s="5" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="K161" s="5" t="n"/>
+      <c r="L161" s="5" t="n"/>
+      <c r="M161" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="N161" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="O161" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P161" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q161" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="R161" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="S161" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="T161" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="U161" s="5" t="n">
+        <v>379</v>
+      </c>
+      <c r="V161" s="5" t="n">
+        <v>394</v>
+      </c>
+      <c r="W161" s="5" t="n">
+        <v>302</v>
+      </c>
+      <c r="X161" s="5" t="n">
+        <v>306</v>
+      </c>
+      <c r="Y161" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z161" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA161" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="AB161" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="AC161" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD161" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE161" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG161" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="AH161" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="AI161" s="5" t="n"/>
+      <c r="AJ161" s="5" t="n"/>
+      <c r="AK161" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="AL161" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="AM161" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN161" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO161" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/es/football/match/real-murcia-real-zaragoza/pgbsMOb</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AO141"/>
+  <autoFilter ref="A1:AO161"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO3" r:id="rId2"/>
@@ -27292,6 +29840,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO139" r:id="rId138"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO140" r:id="rId139"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AO161" r:id="rId160"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -31391,7 +33959,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Métricas de Murcia-Zaragoza y Cartagena-Europa y Alcorcón-Huesca y Águilas-Ibiza y Villarreal B-Teruel y Algeciras-Hércules y Castilla-Antequera y Gimnàstic-Atlético Madrileño y Sant Andreu-Torremolinos incorporadas el 20-10-2026 mediante capturas de Sofascore facilitadas por el usuario; comparación del grupo con corte común J7 mientras falta Real Jaén-Rayo Majadahonda</t>
+          <t>Resuelto el 20-10-2026: J8 completa mediante capturas y texto de Sofascore aportados por el usuario. 80 partidos en grupo2_partidos.csv; 77 con xG por tres ausencias antiguas.</t>
         </is>
       </c>
     </row>
@@ -31551,7 +34119,7 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Faltan los diez partidos de J8: no se presenta la cobertura como actualizada</t>
+          <t>Resuelto el 20-10-2026: J8 completa mediante capturas y texto de Sofascore aportados por el usuario. 80 partidos en grupo2_partidos.csv; 77 con xG por tres ausencias antiguas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excluir partidos sin xG de ambos lados de la comparación de puntos esperados
</commit_message>
<xml_diff>
--- a/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
+++ b/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'clasificacion'!$A$1:$K$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'proximos'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'partidos_rivales'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'goles_video'!$A$1:$Z$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'resumenes_youtube'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'jugadores'!$A$1:$I$26</definedName>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19">
@@ -34128,7 +34128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35199,8 +35199,28 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>xPts sin xG</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Sustituir el xPts ausente por puntos reales oculta la ausencia y mezcla datos con resultados</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Corregido 20-10-2026: xPts queda ausente. Se comparan solo puntos reales y esperados de los mismos partidos con xG; cobertura 7/8 para Huesca y Sant Andreu.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D53"/>
+  <autoFilter ref="A1:D54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza la TV de la jornada 9 y retira la J7 del calendario
</commit_message>
<xml_diff>
--- a/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
+++ b/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'clasificacion'!$A$1:$K$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'proximos'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'partidos_rivales'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'goles_video'!$A$1:$Z$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'resumenes_youtube'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'jugadores'!$A$1:$I$26</definedName>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19">
@@ -34128,7 +34128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35219,8 +35219,28 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Horario y TV J9</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Sofascore (team/next) daba 25-10 16:00 UTC y aún mostraba la J8 sin jugar; respuesta desactualizada</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Se mantiene 23-10 19:15 UTC (21:15 hora local), confirmado por Movistar Plus+, Aragón Digital y Sport Aragón. TV: solo canales citados en al menos dos fuentes; Orange y Embou, en una sola, no se incluyen.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D54"/>
+  <autoFilter ref="A1:D55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Jornada 9: CE Europa 0-1 Real Zaragoza, previa del Villarreal B y Tableau J9
</commit_message>
<xml_diff>
--- a/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
+++ b/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
@@ -29,23 +29,23 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Diccionario'!$A$1:$E$178</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'partidos'!$A$1:$K$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'goles'!$A$1:$J$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'alineaciones'!$A$1:$C$89</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'cambios'!$A$1:$E$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'tarjetas'!$A$1:$E$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'tiros'!$A$1:$J$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'estadisticas'!$A$1:$G$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'partidos'!$A$1:$K$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'goles'!$A$1:$J$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'alineaciones'!$A$1:$C$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'cambios'!$A$1:$E$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'tarjetas'!$A$1:$E$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'tiros'!$A$1:$J$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'estadisticas'!$A$1:$G$163</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'sofascore'!$A$1:$F$304</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'grupo2_partidos'!$A$1:$AQ$161</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'clasificacion'!$A$1:$K$61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'proximos'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'partidos_rivales'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'proximos'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'partidos_rivales'!$A$1:$H$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'goles_video'!$A$1:$Z$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'resumenes_youtube'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'jugadores'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'minutos_partido'!$A$1:$F$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'minutos_partido'!$A$1:$F$145</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11">
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13">
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18">
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>54</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19">
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -33354,7 +33354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -33399,7 +33399,7 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
@@ -33408,17 +33408,17 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Fuera</t>
+          <t>Casa</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>CE Europa</t>
+          <t>Villarreal B</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -33429,7 +33429,7 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
@@ -33438,7 +33438,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-11-08</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -33448,7 +33448,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Villarreal B</t>
+          <t>SD Huesca</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -33457,42 +33457,11 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Primera Federación</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>2026-11-08</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Casa</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>SD Huesca</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>https://www.fotmob.com/es-419/teams/8394/overview</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
+  <autoFilter ref="A1:F3"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -33504,10 +33473,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -34099,8 +34068,296 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Rayo Majadahonda</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/api/v1/event/16599366/statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Algeciras</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/api/v1/event/16599697/statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>SD Huesca</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>https://www.sofascore.com/api/v1/event/16599875/statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Antequera</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>https://www.fotmob.com/es/teams/161771/overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Atlético Madrileño</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>https://www.fotmob.com/es/teams/161771/overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>UD Ibiza</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>https://www.fotmob.com/es/teams/161771/overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Real Jaén</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>https://www.fotmob.com/es/teams/161771/overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>CD Teruel</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>https://www.fotmob.com/es/teams/161771/overview</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H24"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
@@ -34117,6 +34374,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -34128,7 +34393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35239,8 +35504,168 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Gol</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>La web del club (noticia) y Sport Aragón atribuyen el gol del 80 a Diego González; la ficha oficial del club, FotMob, futboltotal y Aragón Digital lo dan en propia puerta de Álex Cano</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Uso la ficha oficial: propia puerta de Álex Cano en el 80 (Sport Aragón da 79 en la crónica). Sin asistencia; el córner lo sacó Rubén Díez</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Aragón Digital empareja Rubén Díez por Ureña (56) y Cuenca por Pereira (78); Sport Aragón da 55 y 77</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Uso la ficha oficial, que coincide con futboltotal: Rubén Díez por Saidu y Pau Sans por Ureña (56), Joaquín por Ander (65), Tobajas por Pereira y Cuenca por Jardí (78); los minutos jugados no cambian</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Tiros</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Ficha oficial: 9-8 tiros y 2-1 a puerta, con desglose que no suma; 365Scores: 10-8 y 3-1. BeSoccer no accesible desde la lectura web (24-10-2026)</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Uso el club y marco el desglose como incompleto; posesión 67-33 coincide en club y 365Scores</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Estadísticas del club</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>La ficha oficial muestra ceros en córners, faltas, tarjetas, paradas y duelos que contradicen los eventos</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>No uso esos ceros; solo posesión y pases. Fueras de juego (2-2) marcados como dudosos</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Sofascore</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Las lecturas web de event/16599975/statistics e incidents fallan, y event/16599975 devolvía el partido sin jugar (24-10-2026)</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Sin métricas de Sofascore ni xG de la J9; queda pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Clasificación</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Solo se ha jugado CE Europa–Real Zaragoza de la J9 (resto, 24 y 25-10). Tabla del club: Zaragoza 1.º con 20 puntos y 9 PJ</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Mantengo clasificacion.csv tras la J8 completa; la tras J9 se añade cuando termine la jornada</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Grupo 2</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>J9 en curso: solo CE Europa–Real Zaragoza terminado (resto, 24 y 25-10); Sofascore no accesible desde la lectura web</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>No añado filas a grupo2_partidos.csv hasta poder leer las estadísticas ALL; el grupo sigue con 80 partidos (J1-J8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Previa Villarreal B</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Futbolme y BeSoccer no accesibles; FotMob solo muestra los cinco últimos partidos (J4-J8)</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>J4-J8 contrastadas entre FotMob y grupo2_partidos.csv (Sofascore); J1-J3 solo Sofascore, con balance total (17-9, 17 puntos) igual a la clasificación oficial tras la J8</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D55"/>
+  <autoFilter ref="A1:D63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -38635,62 +39060,62 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Jaume Jardí</t>
+          <t>Westerveld</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>639</v>
+        <v>720</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>80</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Westerveld</t>
+          <t>Jaume Jardí</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>630</v>
+        <v>717</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="5" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -38699,13 +39124,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>612</v>
+        <v>702</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>2</v>
@@ -38717,10 +39142,10 @@
         <v>2</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.29</v>
+        <v>0.26</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>306</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5">
@@ -38730,13 +39155,13 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C5" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>7</v>
-      </c>
       <c r="D5" s="5" t="n">
-        <v>606</v>
+        <v>696</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>0</v>
@@ -38759,13 +39184,13 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>601</v>
+        <v>691</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>1</v>
@@ -38777,10 +39202,10 @@
         <v>2</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.3</v>
+        <v>0.26</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>300</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7">
@@ -38790,13 +39215,13 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>528</v>
+        <v>618</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>0</v>
@@ -38815,17 +39240,17 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>P. Ademo</t>
+          <t>Raúl Pereira</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>496</v>
+        <v>521</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>0</v>
@@ -38844,17 +39269,17 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Raúl Pereira</t>
+          <t>P. Ademo</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
         <v>7</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>443</v>
+        <v>496</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>0</v>
@@ -38873,62 +39298,62 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Joaquín</t>
+          <t>Óscar Ureña</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>366</v>
+        <v>419</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="4" t="n"/>
+        <v>0.86</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Óscar Ureña</t>
+          <t>Joaquín</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
         <v>7</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>363</v>
+        <v>391</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>91</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -38937,13 +39362,13 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>354</v>
+        <v>388</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>0</v>
@@ -38955,10 +39380,10 @@
         <v>1</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>354</v>
+        <v>388</v>
       </c>
     </row>
     <row r="13">
@@ -38968,13 +39393,13 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>300</v>
+        <v>334</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>1</v>
@@ -38986,55 +39411,57 @@
         <v>1</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0.3</v>
+        <v>0.27</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>300</v>
+        <v>334</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Iker Vadillo</t>
+          <t>Edu Espiau</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>294</v>
+        <v>331</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="4" t="n"/>
+        <v>1.36</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>66</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>S. Escudero</t>
+          <t>Ander Herrera</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>292</v>
+        <v>313</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>0</v>
@@ -39053,17 +39480,17 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Ander Herrera</t>
+          <t>Iker Vadillo</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C16" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="D16" s="4" t="n">
-        <v>248</v>
+        <v>294</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>0</v>
@@ -39082,33 +39509,31 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Edu Espiau</t>
+          <t>S. Escudero</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>3</v>
-      </c>
       <c r="D17" s="5" t="n">
-        <v>241</v>
+        <v>292</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>1.87</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>48</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -39142,53 +39567,57 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>H. Barrachina</t>
+          <t>Yussif Saidu</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>168</v>
+        <v>187</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>187</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Yussif Saidu</t>
+          <t>H. Barrachina</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>168</v>
+      </c>
+      <c r="E20" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>131</v>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="F20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
@@ -39200,13 +39629,13 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C21" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="E21" s="5" t="n">
         <v>0</v>
@@ -39277,17 +39706,17 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Diego Monzón</t>
+          <t>J. Tobajas</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E24" s="4" t="n">
         <v>0</v>
@@ -39304,7 +39733,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>J. Tobajas</t>
+          <t>Diego Monzón</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
@@ -39367,7 +39796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42482,8 +42911,392 @@
         <v>5</v>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>Westerveld</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="F130" s="4" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Marco Sangalli</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="F131" s="5" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>Rubo</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E132" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="F132" s="4" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Diego González</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="F133" s="5" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>Raúl Pereira</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="F134" s="4" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>Lucas Terrer</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="F135" s="5" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>Ander Herrera</t>
+        </is>
+      </c>
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E136" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="F136" s="4" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>Yussif Saidu</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="F137" s="5" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>Jaume Jardí</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="F138" s="4" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Óscar Ureña</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E139" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="F139" s="5" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>Edu Espiau</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E140" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="F140" s="4" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>Rubén Díez</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>Suplente</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="E141" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="F141" s="5" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>Pau Sans</t>
+        </is>
+      </c>
+      <c r="C142" s="4" t="inlineStr">
+        <is>
+          <t>Suplente</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="E142" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="F142" s="4" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Joaquín</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>Suplente</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="E143" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="F143" s="5" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>J. Tobajas</t>
+        </is>
+      </c>
+      <c r="C144" s="4" t="inlineStr">
+        <is>
+          <t>Suplente</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="E144" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="F144" s="4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>Marcos Cuenca</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>Suplente</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="E145" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="F145" s="5" t="n">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F129"/>
+  <autoFilter ref="A1:F145"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -45551,7 +46364,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -45605,7 +46418,7 @@
       </c>
       <c r="E115" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-31</t>
         </is>
       </c>
     </row>
@@ -45632,7 +46445,7 @@
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>Fuera</t>
+          <t>Casa</t>
         </is>
       </c>
     </row>
@@ -45659,7 +46472,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t>CE Europa</t>
+          <t>Villarreal B</t>
         </is>
       </c>
     </row>
@@ -46928,7 +47741,7 @@
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>Jaume Jardí</t>
+          <t>Westerveld</t>
         </is>
       </c>
     </row>
@@ -46982,7 +47795,7 @@
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -47009,7 +47822,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t>639</t>
+          <t>720</t>
         </is>
       </c>
     </row>
@@ -47036,7 +47849,7 @@
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -47063,7 +47876,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -47090,7 +47903,7 @@
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -47117,7 +47930,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>0.0</t>
         </is>
       </c>
     </row>
@@ -47144,7 +47957,7 @@
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -47322,7 +48135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -47755,8 +48568,53 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Primera Federación</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>CE Europa</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K9"/>
+  <autoFilter ref="A1:K10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -47766,6 +48624,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -47777,7 +48636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48924,8 +49783,48 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Álex Cano</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J27"/>
+  <autoFilter ref="A1:J28"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -48953,6 +49852,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -48964,7 +49864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50309,8 +51209,173 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Westerveld</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Marco Sangalli</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Rubo</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Diego González</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Raúl Pereira</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Lucas Terrer</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Ander Herrera</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Yussif Saidu</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>Jaume Jardí</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Óscar Ureña</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Edu Espiau</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C89"/>
+  <autoFilter ref="A1:C100"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -50400,6 +51465,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId99"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -50411,7 +51487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51368,8 +52444,123 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Rubén Díez</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Yussif Saidu</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Pau Sans</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Óscar Ureña</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Joaquín</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Ander Herrera</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>J. Tobajas</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Raúl Pereira</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B46" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Marcos Cuenca</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Jaume Jardí</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E41"/>
+  <autoFilter ref="A1:E46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -51411,6 +52602,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -51422,7 +52618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52057,8 +53253,54 @@
         <v>87</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Lucas Terrer</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Amarilla</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>J. Tobajas</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Amarilla</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>92</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E29"/>
+  <autoFilter ref="A1:E31"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -52088,6 +53330,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -52099,7 +53343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52109,7 +53353,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="43" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
@@ -52484,8 +53728,48 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Web del club (posesión igual en 365Scores)</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>El club da 2 a puerta + 5 fuera + 0 bloqueados (no suman 9); 365Scores da 10-8 tiros y 3-1 a puerta</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J9"/>
+  <autoFilter ref="A1:J10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -52495,6 +53779,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -52506,7 +53791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G159"/>
+  <dimension ref="A1:G163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57453,8 +58738,132 @@
         </is>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>Partido</t>
+        </is>
+      </c>
+      <c r="C160" s="4" t="inlineStr">
+        <is>
+          <t>posesion_pct</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="E160" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="F160" s="4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G160" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>Partido</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>pases</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="n">
+        <v>677</v>
+      </c>
+      <c r="E161" s="5" t="n">
+        <v>330</v>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G161" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>Partido</t>
+        </is>
+      </c>
+      <c r="C162" s="4" t="inlineStr">
+        <is>
+          <t>pases_completados</t>
+        </is>
+      </c>
+      <c r="D162" s="4" t="n">
+        <v>596</v>
+      </c>
+      <c r="E162" s="4" t="n">
+        <v>237</v>
+      </c>
+      <c r="F162" s="4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G162" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>Partido</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>fueras_juego</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E163" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>dudosa</t>
+        </is>
+      </c>
+      <c r="G163" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-primera-federacion-9-ce-europa-vs-real-zaragoza-3940</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G159"/>
+  <autoFilter ref="A1:G163"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -57614,6 +59023,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G157" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G158" r:id="rId157"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G163" r:id="rId162"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Jornada 9: análisis del partido con la revisión del resumen en vídeo
</commit_message>
<xml_diff>
--- a/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
+++ b/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'clasificacion'!$A$1:$K$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'proximos'!$A$1:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'partidos_rivales'!$A$1:$H$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'goles_video'!$A$1:$Z$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'resumenes_youtube'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'jugadores'!$A$1:$I$26</definedName>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19">
@@ -34393,7 +34393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35664,8 +35664,48 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Libro con extracciones hasta J8</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Actualizadas las cuatro extracciones Hyper y el Excel interno a J9 con actualizar_tableau.py (comprobaciones ya no fijas en la J8): 9 partidos, 25 jugadores, 20 equipos (clasificación tras la J8) y 27 goles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Vídeo y ocasiones</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Aragón Digital describe un tiro de Flavio al palo en el 10; Aragón Play, un disparo fuera en el 11; la ficha marca cero al palo (campo poco fiable)</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>No se afirma el palo: se cita solo un disparo de Flavio en torno al 10. Revisión por secuencias del resumen (6:11) aportada por el usuario el 24-10-2026, sin minuto asignado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D63"/>
+  <autoFilter ref="A1:D65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Clasificación y resultados del grupo tras la jornada 9, TV de la Copa y fecha del derbi
</commit_message>
<xml_diff>
--- a/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
+++ b/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
@@ -38,10 +38,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'estadisticas'!$A$1:$G$163</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'sofascore'!$A$1:$F$304</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'grupo2_partidos'!$A$1:$AQ$161</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'clasificacion'!$A$1:$K$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'clasificacion'!$A$1:$K$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'proximos'!$A$1:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'partidos_rivales'!$A$1:$H$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'goles_video'!$A$1:$Z$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'resumenes_youtube'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'jugadores'!$A$1:$I$26</definedName>
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16">
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19">
@@ -30867,7 +30867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33280,8 +33280,788 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B62" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="I62" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J62" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="K62" s="6" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Real Zaragoza</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E63" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F63" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G63" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="I63" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J63" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B64" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Real Jaén</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F64" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="I64" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J64" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K64" s="6" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Real Murcia</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E65" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F65" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H65" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="I65" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="J65" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="K65" s="7" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B66" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Cartagena</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H66" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="I66" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J66" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="K66" s="6" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B67" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Alcorcón</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E67" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F67" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G67" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="I67" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="J67" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B68" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Gimnàstic</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H68" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="I68" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="J68" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="K68" s="6" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B69" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>UD Ibiza</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E69" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F69" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G69" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H69" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="I69" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="J69" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B70" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Algeciras</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F70" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H70" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="I70" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="J70" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="K70" s="6" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B71" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Hércules</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E71" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F71" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H71" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="I71" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="J71" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B72" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>SD Huesca</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E72" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F72" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="I72" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="J72" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="K72" s="6" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B73" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Real Madrid Castilla</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E73" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F73" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G73" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H73" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="I73" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="J73" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="K73" s="7" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B74" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Antequera</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H74" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="I74" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="J74" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K74" s="6" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B75" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Atlético Madrileño</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E75" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G75" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H75" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="I75" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="J75" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="K75" s="7" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B76" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Sant Andreu</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F76" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G76" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H76" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I76" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="J76" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K76" s="6" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B77" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Rayo Majadahonda</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E77" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F77" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H77" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="I77" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J77" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="K77" s="7" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B78" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>CDA Águilas FC</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E78" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G78" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H78" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="I78" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="J78" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K78" s="6" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B79" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>CE Europa</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E79" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F79" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H79" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I79" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="J79" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="K79" s="7" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B80" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Juventud Torremolinos CF</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F80" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G80" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H80" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="I80" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J80" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K80" s="6" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B81" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>CD Teruel</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E81" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G81" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H81" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I81" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="J81" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K81" s="7" t="inlineStr">
+        <is>
+          <t>https://es.besoccer.com/competicion/clasificacion/primera_division_rfef/2027/grupo2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K61"/>
+  <autoFilter ref="A1:K81"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -33343,6 +34123,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -33438,7 +34238,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>2026-11-08</t>
+          <t>2026-11-07</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -34393,7 +35193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35704,8 +36504,88 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Clasificación</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>J9 completa el 25-10. BeSoccer (tabla tras la J9) coincide con la clasificación tras la J8 más los diez resultados de la J9 (El Periódico de Ceuta)</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Añadida la clasificación tras la J9 con el orden de BeSoccer (Huesca 11.º y Castilla 12.º, empatados en puntos, diferencia y goles)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Grupo 2</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>J9 completa (10 resultados, El Periódico de Ceuta, cuadran con BeSoccer); Sofascore sigue sin responder a la lectura web</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Añadidos los resultados a grupo2_resultados.csv; grupo2_partidos.csv sigue con J1-J8 (80 partidos) hasta poder leer las estadísticas ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Calendario</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>proximos.csv tenía el Real Zaragoza-SD Huesca el 08-11; la RFEF fijó el sábado 07-11 a las 21:00 (Sport Aragón 15-10, futboltotal y datos/sofascore.json)</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Corregida la fecha a 2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>TV Copa</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>CD Tudelano-Real Zaragoza (27-10, 21:00, Municipal de Tudela): Aragón TV en abierto según Sport Aragón (26-10) y Aragón Digital (21-10)</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Añadido Aragón TV (abierto) a la lista tv de datos/sofascore.json</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D65"/>
+  <autoFilter ref="A1:D69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Añade CD Tudelano 0-4 (Copa) y previa en redes de la J10
</commit_message>
<xml_diff>
--- a/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
+++ b/analisis/real-zaragoza/datos/tablas/datos_real_zaragoza.xlsx
@@ -29,10 +29,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Diccionario'!$A$1:$E$178</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'partidos'!$A$1:$K$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'goles'!$A$1:$J$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'alineaciones'!$A$1:$C$100</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'cambios'!$A$1:$E$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'partidos'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'goles'!$A$1:$J$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'alineaciones'!$A$1:$C$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'cambios'!$A$1:$E$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'tarjetas'!$A$1:$E$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'tiros'!$A$1:$J$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'estadisticas'!$A$1:$G$163</definedName>
@@ -40,8 +40,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'grupo2_partidos'!$A$1:$AQ$161</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'clasificacion'!$A$1:$K$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'proximos'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'partidos_rivales'!$A$1:$H$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'partidos_rivales'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'incidencias'!$A$1:$D$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'goles_video'!$A$1:$Z$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'resumenes_youtube'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'jugadores'!$A$1:$I$26</definedName>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8">
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>99</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18">
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19">
@@ -34273,7 +34273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35156,8 +35156,44 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Villarreal B</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Cartagena</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>https://www.elperiodicodeceuta.es/resultados-primera-federacion-grupo-2-jornada-9-2026-27/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H24"/>
+  <autoFilter ref="A1:H25"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
@@ -35182,6 +35218,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -35193,7 +35230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -36584,8 +36621,148 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Goles</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Minutos de los goles: ficha del club 12', 20' (penalti), 37' y 41'; Aragón Digital y Sport Aragón 11', 19', 36' y 40'. futboltotal da los dos goles de Pau Sans de penalti; el club, Aragón Digital y Sport Aragón solo el primero</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Se usan los minutos del club y solo el 0-2 como penalti</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Asistencias</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Solo la ficha del club da asistencia (Marcos Cuenca en el 0-1). Aragón Digital describe un pase de Pau Sans en el 0-4 que el club no registra como asistencia</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Se apunta solo la asistencia del club</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Cambios</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Primer cambio del Zaragoza (Escudero por Raúl Pereira): 45' en la ficha del club, 46' en Aragón Digital y futboltotal; entra tras el descanso</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Se apunta en el 46'</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Estadísticas</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>La ficha del club muestra ceros en todas las estadísticas del partido; Sport Aragón y Aragón Digital no publican estadísticas; Sofascore no responde desde la lectura web (client_error)</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Sin tiros, posesión ni estadísticas: se dejan vacías</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Tarjetas</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Ninguna tarjeta al Zaragoza en el club, Aragón Digital y futboltotal. La única amarilla es del Tudelano (Olartzabal 47' según el club; el entrenador según Aragón Digital)</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Sin tarjetas del Zaragoza</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Real Zaragoza-Villarreal B: la ficha del club (31-10, 21:00, Ibercaja Estadio) y futbolenlatele coinciden; FotMob lo lista el domingo 1-11 a las 16:00 y el listado de Sofascore también el 1-11, pero ese listado sigue mostrando como no jugadas la J8 y la J9 (copia desactualizada)</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>Se mantiene el sábado 31-10 a las 21:00 (club y futbolenlatele)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>TV</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Solo futbolenlatele indica Aragón TV, Aragón Play y Movistar; el club no publica la emisión y no hay una segunda fuente para este partido</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>tv se deja vacía hasta tener dos fuentes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D69"/>
+  <autoFilter ref="A1:D76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -49055,7 +49232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -49533,8 +49710,51 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Copa del Rey</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Fuera</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>CD Tudelano</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K10"/>
+  <autoFilter ref="A1:K11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -49545,6 +49765,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -49556,7 +49777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50743,8 +50964,172 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Joaquín</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Marcos Cuenca</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Pau Sans</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="n"/>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Pau Sans</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Hugo Pinilla</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J28"/>
+  <autoFilter ref="A1:J32"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -50773,6 +51158,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -50784,7 +51173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52294,8 +52683,173 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Anartz Peña</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>J. Gabilondo</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Raúl Pereira</t>
+        </is>
+      </c>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>H. Barrachina</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Tachi</t>
+        </is>
+      </c>
+      <c r="C105" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>Marcos Cuenca</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Hugo Pinilla</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>Yussif Saidu</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Joaquín</t>
+        </is>
+      </c>
+      <c r="C109" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>Diego Monzón</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Pau Sans</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C100"/>
+  <autoFilter ref="A1:C111"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -52396,6 +52950,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -52407,7 +52972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -53479,8 +54044,123 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>S. Escudero</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Raúl Pereira</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B48" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Lalo Arantegui</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>J. Gabilondo</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>J. Tobajas</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Pau Sans</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B50" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Laken Torres</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Joaquín</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Sergio Beltrán</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Diego Monzón</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>https://www.realzaragoza.com/partidos/temporada-2026-2027-copa-del-rey-3-tudelano-vs-real-zaragoza-5218</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E46"/>
+  <autoFilter ref="A1:E51"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -53527,6 +54207,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>